<commit_message>
Fixed the updated issue
</commit_message>
<xml_diff>
--- a/src/data/TAHERI_SCOUT_BAND_GROUP_1448H.xlsx
+++ b/src/data/TAHERI_SCOUT_BAND_GROUP_1448H.xlsx
@@ -1544,7 +1544,7 @@
         <v>40915293</v>
       </c>
       <c r="C40" t="str">
-        <v>ALIASGAR MUFADDAL KANCHWALA</v>
+        <v>ALIASGAR MUFADDALBHAI KANCHWALA</v>
       </c>
       <c r="D40" t="str">
         <v>Idries manjil 3rd floor noor baugh</v>
@@ -1556,7 +1556,7 @@
         <v>SHUJAI SECTOR</v>
       </c>
       <c r="G40" t="str">
-        <v>Trumpet Member</v>
+        <v>Ghugara Member</v>
       </c>
       <c r="H40" t="str">
         <v>aliasgarKanchwala@tsgband.com</v>
@@ -2744,7 +2744,7 @@
         <v>40915293</v>
       </c>
       <c r="C40" t="str">
-        <v>ALIASGAR MUFADDAL KANCHWALA</v>
+        <v>ALIASGAR MUFADDALBHAI KANCHWALA</v>
       </c>
       <c r="D40" t="str">
         <v>Idries manjil 3rd floor noor baugh</v>
@@ -2756,7 +2756,7 @@
         <v>SHUJAI SECTOR</v>
       </c>
       <c r="G40" t="str">
-        <v>Trumpet Member</v>
+        <v>Ghugara Member</v>
       </c>
       <c r="H40" t="str">
         <v>aliasgarKanchwala@tsgband.com</v>
@@ -3236,7 +3236,7 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>ALIASGAR MUFADDAL KANCHWALA</v>
+        <v>ALIASGAR MUFADDALBHAI KANCHWALA</v>
       </c>
       <c r="B40" t="str">
         <v/>
@@ -3676,7 +3676,7 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>ALIASGAR MUFADDAL KANCHWALA</v>
+        <v>ALIASGAR MUFADDALBHAI KANCHWALA</v>
       </c>
       <c r="B38" t="str">
         <v>Lavajam</v>

</xml_diff>

<commit_message>
Fixed the ss issue
</commit_message>
<xml_diff>
--- a/src/data/TAHERI_SCOUT_BAND_GROUP_1448H.xlsx
+++ b/src/data/TAHERI_SCOUT_BAND_GROUP_1448H.xlsx
@@ -3830,7 +3830,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3890,9 +3890,38 @@
         <v>BURHAN JUZARBHAI KUNDAWALA (Trumpet Major)</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2026-09-29T12:26:22.191Z</v>
+      </c>
+      <c r="B3" t="str">
+        <v>AQA Moula Tune</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Trumpet</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Trumpet Notes</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Aqa Moula Converted.pdf</v>
+      </c>
+      <c r="F3" t="str">
+        <v>/uploads/tunes/Trumpet%20Notes/1790684782183_Aqa_Moula_Converted.pdf</v>
+      </c>
+      <c r="G3" t="str">
+        <v>https://www.youtube.com/watch?v=fRhv0VRICr0</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>BURHAN JUZARBHAI KUNDAWALA (Trumpet Major)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>